<commit_message>
Ajusta relatorio preliminar e matriz de achados
</commit_message>
<xml_diff>
--- a/02-Execucao/01-Questionario/iGovTI-2026.xlsx
+++ b/02-Execucao/01-Questionario/iGovTI-2026.xlsx
@@ -1,44 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\CAD-TI\SERVIDORES\Augusto\workspace\tcerj-igovti-2026\02-Execucao\01-Questionario\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F90DD4F0-8D8D-4C1F-B3C2-97C2659D4161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
+    <workbookView xWindow="-18390" yWindow="3090" windowWidth="12585" windowHeight="12480" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="resultados" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="resultados" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="131">
   <si>
     <t>sigla</t>
   </si>
@@ -46,9 +28,6 @@
     <t>iGovTI</t>
   </si>
   <si>
-    <t>nivel_maturidade</t>
-  </si>
-  <si>
     <t>GovernancaTI</t>
   </si>
   <si>
@@ -154,7 +133,7 @@
     <t>INEA</t>
   </si>
   <si>
-    <t xml:space="preserve">DUQUE DE CAXIAS</t>
+    <t>DUQUE DE CAXIAS</t>
   </si>
   <si>
     <t>RIOTRILHOS</t>
@@ -184,7 +163,7 @@
     <t>FAPERJ</t>
   </si>
   <si>
-    <t xml:space="preserve">CASIMIRO DE ABREU</t>
+    <t>CASIMIRO DE ABREU</t>
   </si>
   <si>
     <t>ARARUAMA</t>
@@ -193,7 +172,7 @@
     <t>QUISSAMÃ</t>
   </si>
   <si>
-    <t xml:space="preserve">PORTO REAL</t>
+    <t>PORTO REAL</t>
   </si>
   <si>
     <t>PRODERJ</t>
@@ -262,16 +241,16 @@
     <t>SEENEMAR</t>
   </si>
   <si>
-    <t xml:space="preserve">SÃO PEDRO DA ALDEIA</t>
+    <t>SÃO PEDRO DA ALDEIA</t>
   </si>
   <si>
     <t>IEEA</t>
   </si>
   <si>
-    <t xml:space="preserve">RIO DAS OSTRAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NOVA FRIBURGO</t>
+    <t>RIO DAS OSTRAS</t>
+  </si>
+  <si>
+    <t>NOVA FRIBURGO</t>
   </si>
   <si>
     <t>SEPM</t>
@@ -289,13 +268,13 @@
     <t>CENTRAL</t>
   </si>
   <si>
-    <t xml:space="preserve">ARMAÇÃO DOS BÚZIOS</t>
+    <t>ARMAÇÃO DOS BÚZIOS</t>
   </si>
   <si>
     <t>RIOPREVIDENCIA</t>
   </si>
   <si>
-    <t xml:space="preserve">SÃO JOÃO DE MERITI</t>
+    <t>SÃO JOÃO DE MERITI</t>
   </si>
   <si>
     <t>TJRJ</t>
@@ -307,16 +286,16 @@
     <t>CEASA</t>
   </si>
   <si>
-    <t xml:space="preserve">CABO FRIO</t>
+    <t>CABO FRIO</t>
   </si>
   <si>
     <t>SEFAZ</t>
   </si>
   <si>
-    <t xml:space="preserve">BELFORD ROXO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SÃO JOÃO DA BARRA</t>
+    <t>BELFORD ROXO</t>
+  </si>
+  <si>
+    <t>SÃO JOÃO DA BARRA</t>
   </si>
   <si>
     <t>PARATY</t>
@@ -331,10 +310,10 @@
     <t>GSI</t>
   </si>
   <si>
-    <t xml:space="preserve">NOVA IGUAÇU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VOLTA REDONDA</t>
+    <t>NOVA IGUAÇU</t>
+  </si>
+  <si>
+    <t>VOLTA REDONDA</t>
   </si>
   <si>
     <t>DETRAN</t>
@@ -343,7 +322,7 @@
     <t>SEIJES</t>
   </si>
   <si>
-    <t xml:space="preserve">ARRAIAL DO CABO</t>
+    <t>ARRAIAL DO CABO</t>
   </si>
   <si>
     <t>LOTERJ</t>
@@ -385,13 +364,13 @@
     <t>UERJ</t>
   </si>
   <si>
-    <t xml:space="preserve">BARRA DO PIRAÍ</t>
+    <t>BARRA DO PIRAÍ</t>
   </si>
   <si>
     <t>MPERJ</t>
   </si>
   <si>
-    <t xml:space="preserve">ANGRA DOS REIS</t>
+    <t>ANGRA DOS REIS</t>
   </si>
   <si>
     <t>TCE-RJ</t>
@@ -421,7 +400,7 @@
     <t>FS</t>
   </si>
   <si>
-    <t xml:space="preserve">SÃO GONÇALO</t>
+    <t>SÃO GONÇALO</t>
   </si>
   <si>
     <t>EMATER</t>
@@ -431,17 +410,27 @@
   </si>
   <si>
     <t>ISP</t>
+  </si>
+  <si>
+    <t>iGovTI_maturidade</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="12.000000"/>
+      <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -455,18 +444,19 @@
   </fills>
   <borders count="1">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,295 +467,15 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
   </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
-  <a:themeElements>
-    <a:clrScheme name="Office">
-      <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="1F497D"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="EEECE1"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="4F81BD"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="C0504D"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="9BBB59"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8064A2"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="4BACC6"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="F79646"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000FF"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="800080"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Cambria"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Angsana New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface=""/>
-        <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ 明朝"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Cordia New"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme name="Office">
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="50000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="35000">
-              <a:schemeClr val="phClr">
-                <a:tint val="37000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="80000">
-              <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
-                <a:satMod val="130000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
-                <a:satMod val="135000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
-        </a:gradFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
-              <a:satMod val="105000"/>
-            </a:schemeClr>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="38000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="35000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
-          <a:scene3d>
-            <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
-            </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
-            </a:lightRig>
-          </a:scene3d>
-          <a:sp3d>
-            <a:bevelT w="63500" h="25400"/>
-          </a:sp3d>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="40000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="40000">
-              <a:schemeClr val="phClr">
-                <a:tint val="45000"/>
-                <a:shade val="99000"/>
-                <a:satMod val="350000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
-                <a:satMod val="255000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
-          </a:path>
-        </a:gradFill>
-        <a:gradFill rotWithShape="1">
-          <a:gsLst>
-            <a:gs pos="0">
-              <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
-                <a:satMod val="300000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="100000">
-              <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
-                <a:satMod val="200000"/>
-              </a:schemeClr>
-            </a:gs>
-          </a:gsLst>
-          <a:path path="circle">
-            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
-          </a:path>
-        </a:gradFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
-</a:theme>
-</file>
-
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:p="http://schemas.openxmlformats.org/presentationml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1016,76 +726,78 @@
       </a:style>
     </a:lnDef>
   </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:M116"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="1" max="2" width="14.83203125"/>
-    <col customWidth="1" min="3" max="3" width="18.83203125"/>
-    <col customWidth="1" min="4" max="4" width="14.83203125"/>
-    <col customWidth="1" min="5" max="5" width="16.83203125"/>
-    <col customWidth="1" min="6" max="6" width="14.83203125"/>
-    <col customWidth="1" min="7" max="7" width="17.83203125"/>
-    <col customWidth="1" min="8" max="8" width="18.83203125"/>
-    <col customWidth="1" min="9" max="9" width="19.83203125"/>
-    <col customWidth="1" min="10" max="10" width="14.83203125"/>
-    <col customWidth="1" min="11" max="12" width="17.83203125"/>
-    <col customWidth="1" min="13" max="13" width="14.83203125"/>
+    <col min="1" max="2" width="14.875" customWidth="1"/>
+    <col min="3" max="3" width="18.875" customWidth="1"/>
+    <col min="4" max="4" width="14.875" customWidth="1"/>
+    <col min="5" max="5" width="16.875" customWidth="1"/>
+    <col min="6" max="6" width="14.875" customWidth="1"/>
+    <col min="7" max="7" width="17.875" customWidth="1"/>
+    <col min="8" max="8" width="18.875" customWidth="1"/>
+    <col min="9" max="9" width="19.875" customWidth="1"/>
+    <col min="10" max="10" width="14.875" customWidth="1"/>
+    <col min="11" max="12" width="17.875" customWidth="1"/>
+    <col min="13" max="13" width="14.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
+      <c r="B2">
+        <v>2.5201767888585858E-2</v>
+      </c>
+      <c r="C2" t="s">
         <v>13</v>
-      </c>
-      <c r="B2">
-        <v>0.025201767888585858</v>
-      </c>
-      <c r="C2" t="s">
-        <v>14</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1115,18 +827,18 @@
         <v>0.13580761609141043</v>
       </c>
       <c r="M2">
-        <v>0.048251176186518682</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>4.8251176186518682E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3">
         <v>0.17485127253273761</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3">
         <v>0.22315378057725038</v>
@@ -1135,13 +847,13 @@
         <v>0.20695156753110971</v>
       </c>
       <c r="F3">
-        <v>0.037800598936254752</v>
+        <v>3.7800598936254752E-2</v>
       </c>
       <c r="G3">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="H3">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="I3">
         <v>0.5</v>
@@ -1153,33 +865,33 @@
         <v>0.37314627825785823</v>
       </c>
       <c r="L3">
-        <v>0.049999999999999947</v>
+        <v>4.9999999999999947E-2</v>
       </c>
       <c r="M3">
         <v>0.13067404517892151</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4">
-        <v>0.088841594119021122</v>
+        <v>8.8841594119021122E-2</v>
       </c>
       <c r="C4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D4">
         <v>0.10864756287475605</v>
       </c>
       <c r="E4">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F4">
-        <v>0.074039373928800001</v>
+        <v>7.4039373928800001E-2</v>
       </c>
       <c r="G4">
-        <v>0.0502282515626283</v>
+        <v>5.02282515626283E-2</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -1194,21 +906,21 @@
         <v>0.14060407834502253</v>
       </c>
       <c r="L4">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M4">
-        <v>0.070727156171443817</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>7.0727156171443817E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5">
         <v>0.22121734589147629</v>
       </c>
       <c r="C5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D5">
         <v>0.11515332291697254</v>
@@ -1229,7 +941,7 @@
         <v>0.5</v>
       </c>
       <c r="J5">
-        <v>0.083333333333333495</v>
+        <v>8.3333333333333495E-2</v>
       </c>
       <c r="K5">
         <v>0.22959520069749167</v>
@@ -1241,15 +953,15 @@
         <v>0.31822296002412209</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>0.19143433660338052</v>
       </c>
       <c r="C6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D6">
         <v>0.15404076441367928</v>
@@ -1264,16 +976,16 @@
         <v>0.29941349495233777</v>
       </c>
       <c r="H6">
-        <v>0.069567866188854605</v>
+        <v>6.9567866188854605E-2</v>
       </c>
       <c r="I6">
         <v>0</v>
       </c>
       <c r="J6">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K6">
-        <v>0.064127204543256516</v>
+        <v>6.4127204543256516E-2</v>
       </c>
       <c r="L6">
         <v>0.23587625194001161</v>
@@ -1282,15 +994,15 @@
         <v>0.22563430689629849</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>0.26459593198887882</v>
       </c>
       <c r="C7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D7">
         <v>0.1216576931116455</v>
@@ -1317,33 +1029,33 @@
         <v>0.28649735037772284</v>
       </c>
       <c r="L7">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M7">
         <v>0.39532651580482547</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>0.13668038450360992</v>
       </c>
       <c r="C8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D8">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="E8">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F8">
         <v>0.11340179680876425</v>
       </c>
       <c r="G8">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H8">
         <v>0</v>
@@ -1364,15 +1076,15 @@
         <v>0.12449833214502061</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>0.32199204935215442</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D9">
         <v>0.20589593578186027</v>
@@ -1384,7 +1096,7 @@
         <v>0.29870248643542052</v>
       </c>
       <c r="G9">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H9">
         <v>0.73200914076079049</v>
@@ -1405,15 +1117,15 @@
         <v>0.42817296234662944</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B10">
-        <v>0.073470340584407531</v>
+        <v>7.3470340584407531E-2</v>
       </c>
       <c r="C10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D10">
         <v>0</v>
@@ -1425,7 +1137,7 @@
         <v>0.11383779882519196</v>
       </c>
       <c r="G10">
-        <v>0.097265825310939594</v>
+        <v>9.7265825310939594E-2</v>
       </c>
       <c r="H10">
         <v>0.16103305013004807</v>
@@ -1446,15 +1158,15 @@
         <v>0.1406659391394269</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>0.37644491826924709</v>
       </c>
       <c r="C11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D11">
         <v>0.54715909751347569</v>
@@ -1469,7 +1181,7 @@
         <v>0.36347006914117025</v>
       </c>
       <c r="H11">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -1487,15 +1199,15 @@
         <v>0.22031060114346912</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>0.29591377320585005</v>
       </c>
       <c r="C12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D12">
         <v>0.25040021093861525</v>
@@ -1528,15 +1240,15 @@
         <v>0.33754024498468166</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>0.20892874272585549</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D13">
         <v>0.11725961651480429</v>
@@ -1548,7 +1260,7 @@
         <v>0.23295592723346767</v>
       </c>
       <c r="G13">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H13">
         <v>0.389984841777339</v>
@@ -1569,18 +1281,18 @@
         <v>0.2927688577405731</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>0.10721629504052509</v>
       </c>
       <c r="C14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D14">
-        <v>0.049110575227793551</v>
+        <v>4.9110575227793551E-2</v>
       </c>
       <c r="E14">
         <v>0.28879088425724181</v>
@@ -1592,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>0.052937832745001252</v>
+        <v>5.2937832745001252E-2</v>
       </c>
       <c r="I14">
         <v>0</v>
@@ -1610,15 +1322,15 @@
         <v>0.16035948984851783</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B15">
         <v>0.48669509529632521</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15">
         <v>0.478252794103597</v>
@@ -1651,30 +1363,30 @@
         <v>0.49441638088333562</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B16">
         <v>0.11163284427283718</v>
       </c>
       <c r="C16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D16">
         <v>0.12696032028653115</v>
       </c>
       <c r="E16">
-        <v>0.025112250804977549</v>
+        <v>2.5112250804977549E-2</v>
       </c>
       <c r="F16">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="G16">
-        <v>0.069476925209936494</v>
+        <v>6.9476925209936494E-2</v>
       </c>
       <c r="H16">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="I16">
         <v>0</v>
@@ -1686,24 +1398,24 @@
         <v>0.19274692069908203</v>
       </c>
       <c r="L16">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M16">
-        <v>0.097614412931898917</v>
-      </c>
-    </row>
-    <row r="17">
+        <v>9.7614412931898917E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B17">
-        <v>0.014585492144573966</v>
+        <v>1.4585492144573966E-2</v>
       </c>
       <c r="C17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D17">
-        <v>0.012165769311164551</v>
+        <v>1.2165769311164551E-2</v>
       </c>
       <c r="E17">
         <v>0.10950609645809879</v>
@@ -1730,33 +1442,33 @@
         <v>0</v>
       </c>
       <c r="M17">
-        <v>0.016798558299363244</v>
-      </c>
-    </row>
-    <row r="18">
+        <v>1.6798558299363244E-2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18">
-        <v>0.065708746110145086</v>
+        <v>6.5708746110145086E-2</v>
       </c>
       <c r="C18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D18">
-        <v>0.089691325097975005</v>
+        <v>8.9691325097975005E-2</v>
       </c>
       <c r="E18">
-        <v>0.025112250804977549</v>
+        <v>2.5112250804977549E-2</v>
       </c>
       <c r="F18">
-        <v>0.036162201174808048</v>
+        <v>3.6162201174808048E-2</v>
       </c>
       <c r="G18">
-        <v>0.016742750520876103</v>
+        <v>1.6742750520876103E-2</v>
       </c>
       <c r="H18">
-        <v>0.01764594424833375</v>
+        <v>1.764594424833375E-2</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -1771,59 +1483,59 @@
         <v>0</v>
       </c>
       <c r="M18">
-        <v>0.043774401758918932</v>
-      </c>
-    </row>
-    <row r="19">
+        <v>4.3774401758918932E-2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>32</v>
+      </c>
+      <c r="B19">
+        <v>4.970205662625881E-2</v>
+      </c>
+      <c r="C19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19">
+        <v>0.05</v>
+      </c>
+      <c r="E19">
+        <v>0.05</v>
+      </c>
+      <c r="F19">
+        <v>0.05</v>
+      </c>
+      <c r="G19">
+        <v>0.05</v>
+      </c>
+      <c r="H19">
+        <v>0.05</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="K19">
+        <v>4.6868026115007511E-2</v>
+      </c>
+      <c r="L19">
+        <v>4.9999999999999947E-2</v>
+      </c>
+      <c r="M19">
+        <v>4.9429559137138826E-2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>33</v>
-      </c>
-      <c r="B19">
-        <v>0.04970205662625881</v>
-      </c>
-      <c r="C19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="E19">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="F19">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="G19">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="H19">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="I19">
-        <v>0</v>
-      </c>
-      <c r="J19">
-        <v>0.041666666666666657</v>
-      </c>
-      <c r="K19">
-        <v>0.046868026115007511</v>
-      </c>
-      <c r="L19">
-        <v>0.049999999999999947</v>
-      </c>
-      <c r="M19">
-        <v>0.049429559137138826</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>34</v>
       </c>
       <c r="B20">
         <v>0.19375139604719799</v>
       </c>
       <c r="C20" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D20">
         <v>0.17824712411953259</v>
@@ -1832,7 +1544,7 @@
         <v>0.36345413184230912</v>
       </c>
       <c r="F20">
-        <v>0.093039787560443371</v>
+        <v>9.3039787560443371E-2</v>
       </c>
       <c r="G20">
         <v>0.25727126543813994</v>
@@ -1856,15 +1568,15 @@
         <v>0.20793152402880649</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B21">
         <v>0.34140848111684408</v>
       </c>
       <c r="C21" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D21">
         <v>0.47598498335888056</v>
@@ -1873,7 +1585,7 @@
         <v>0.80865458681576907</v>
       </c>
       <c r="F21">
-        <v>0.077239595633956201</v>
+        <v>7.7239595633956201E-2</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1897,30 +1609,30 @@
         <v>0.21832549895473721</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B22">
         <v>0.16676128089382131</v>
       </c>
       <c r="C22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D22">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="E22">
         <v>0.14999999999999997</v>
       </c>
       <c r="F22">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="G22">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H22">
-        <v>0.069291806016055627</v>
+        <v>6.9291806016055627E-2</v>
       </c>
       <c r="I22">
         <v>0.5</v>
@@ -1938,27 +1650,27 @@
         <v>0.1820910628609429</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B23">
         <v>0.21149565862143171</v>
       </c>
       <c r="C23" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D23">
         <v>0.13896743477721413</v>
       </c>
       <c r="E23">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="F23">
         <v>0.5036216264259995</v>
       </c>
       <c r="G23">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H23">
         <v>0.18266101678445765</v>
@@ -1979,15 +1691,15 @@
         <v>0.27782960201380713</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B24">
         <v>0.34417805334279772</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>0.21146953542185148</v>
@@ -2020,15 +1732,15 @@
         <v>0.46555258657777809</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B25">
         <v>0.23478371953958638</v>
       </c>
       <c r="C25" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D25">
         <v>0.25342188301506213</v>
@@ -2061,24 +1773,24 @@
         <v>0.21773735034163702</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B26">
-        <v>0.069337088290516768</v>
+        <v>6.9337088290516768E-2</v>
       </c>
       <c r="C26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D26">
-        <v>0.030154337451012501</v>
+        <v>3.0154337451012501E-2</v>
       </c>
       <c r="E26">
         <v>0.32421424436515711</v>
       </c>
       <c r="F26">
-        <v>0.077239595633956201</v>
+        <v>7.7239595633956201E-2</v>
       </c>
       <c r="G26">
         <v>0</v>
@@ -2093,7 +1805,7 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K26">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L26">
         <v>0.14999999999999986</v>
@@ -2102,21 +1814,21 @@
         <v>0.10517343224577339</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B27">
         <v>0.14465260614672573</v>
       </c>
       <c r="C27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>0.075336752414932651</v>
+        <v>7.5336752414932651E-2</v>
       </c>
       <c r="F27">
         <v>0.33084458154155522</v>
@@ -2143,15 +1855,15 @@
         <v>0.2769511415183662</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B28">
         <v>0.50772389047606492</v>
       </c>
       <c r="C28" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D28">
         <v>0.61251913941256453</v>
@@ -2184,15 +1896,15 @@
         <v>0.4118786906036036</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B29">
-        <v>0.014599225313320672</v>
+        <v>1.4599225313320672E-2</v>
       </c>
       <c r="C29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D29">
         <v>0</v>
@@ -2222,18 +1934,18 @@
         <v>0</v>
       </c>
       <c r="M29">
-        <v>0.027951602280202045</v>
-      </c>
-    </row>
-    <row r="30">
+        <v>2.7951602280202045E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B30">
         <v>0.29863825042698661</v>
       </c>
       <c r="C30" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D30">
         <v>0.21588371099682671</v>
@@ -2242,7 +1954,7 @@
         <v>0.68143681030371261</v>
       </c>
       <c r="F30">
-        <v>0.087596183571882452</v>
+        <v>8.7596183571882452E-2</v>
       </c>
       <c r="G30">
         <v>0.13812769179722784</v>
@@ -2266,15 +1978,15 @@
         <v>0.37432512986598965</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B31">
-        <v>0.090830036922830357</v>
+        <v>9.0830036922830357E-2</v>
       </c>
       <c r="C31" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D31">
         <v>0</v>
@@ -2286,7 +1998,7 @@
         <v>0.24038723041216309</v>
       </c>
       <c r="G31">
-        <v>0.052734174689060394</v>
+        <v>5.2734174689060394E-2</v>
       </c>
       <c r="H31">
         <v>0</v>
@@ -2298,24 +2010,24 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K31">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L31">
-        <v>0.076391784051418346</v>
+        <v>7.6391784051418346E-2</v>
       </c>
       <c r="M31">
         <v>0.1739027251566917</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B32">
         <v>0.30923553468549303</v>
       </c>
       <c r="C32" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D32">
         <v>0.27449070333259218</v>
@@ -2348,18 +2060,18 @@
         <v>0.34101298012647502</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B33">
         <v>0.25066746928637917</v>
       </c>
       <c r="C33" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D33">
-        <v>0.03649730793349365</v>
+        <v>3.649730793349365E-2</v>
       </c>
       <c r="E33">
         <v>1</v>
@@ -2389,15 +2101,15 @@
         <v>0.4465464058784665</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B34">
-        <v>0.0065547542223072406</v>
+        <v>6.5547542223072406E-3</v>
       </c>
       <c r="C34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D34">
         <v>0</v>
@@ -2421,68 +2133,68 @@
         <v>0.18333333333333329</v>
       </c>
       <c r="K34">
-        <v>0.06890342546983462</v>
+        <v>6.890342546983462E-2</v>
       </c>
       <c r="L34">
         <v>0</v>
       </c>
       <c r="M34">
-        <v>0.012549698982947858</v>
-      </c>
-    </row>
-    <row r="35">
+        <v>1.2549698982947858E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>48</v>
+      </c>
+      <c r="B35">
+        <v>0</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35">
+        <v>0</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35">
+        <v>0</v>
+      </c>
+      <c r="G35">
+        <v>0</v>
+      </c>
+      <c r="H35">
+        <v>0</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <v>0</v>
+      </c>
+      <c r="K35">
+        <v>0</v>
+      </c>
+      <c r="L35">
+        <v>0</v>
+      </c>
+      <c r="M35">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>49</v>
       </c>
-      <c r="B35">
-        <v>0</v>
-      </c>
-      <c r="C35" t="s">
-        <v>14</v>
-      </c>
-      <c r="D35">
-        <v>0</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35">
-        <v>0</v>
-      </c>
-      <c r="G35">
-        <v>0</v>
-      </c>
-      <c r="H35">
-        <v>0</v>
-      </c>
-      <c r="I35">
-        <v>0</v>
-      </c>
-      <c r="J35">
-        <v>0</v>
-      </c>
-      <c r="K35">
-        <v>0</v>
-      </c>
-      <c r="L35">
-        <v>0</v>
-      </c>
-      <c r="M35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="s">
-        <v>50</v>
-      </c>
       <c r="B36">
-        <v>0.032850833094786848</v>
+        <v>3.2850833094786848E-2</v>
       </c>
       <c r="C36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D36">
-        <v>0.01637019174259785</v>
+        <v>1.637019174259785E-2</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2491,77 +2203,77 @@
         <v>0</v>
       </c>
       <c r="G36">
-        <v>0.032421941770313205</v>
+        <v>3.2421941770313205E-2</v>
       </c>
       <c r="H36">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="I36">
         <v>0</v>
       </c>
       <c r="J36">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K36">
-        <v>0.046868026115007511</v>
+        <v>4.6868026115007511E-2</v>
       </c>
       <c r="L36">
         <v>0.16551553211140643</v>
       </c>
       <c r="M36">
-        <v>0.04792394356932806</v>
-      </c>
-    </row>
-    <row r="37">
+        <v>4.792394356932806E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>50</v>
+      </c>
+      <c r="B37">
+        <v>2.7498017162912278E-3</v>
+      </c>
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37">
+        <v>0</v>
+      </c>
+      <c r="E37">
+        <v>0</v>
+      </c>
+      <c r="F37">
+        <v>0</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>3.336996655614665E-2</v>
+      </c>
+      <c r="I37">
+        <v>0</v>
+      </c>
+      <c r="J37">
+        <v>0</v>
+      </c>
+      <c r="K37">
+        <v>0</v>
+      </c>
+      <c r="L37">
+        <v>0</v>
+      </c>
+      <c r="M37">
+        <v>5.2647563328623529E-3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>51</v>
-      </c>
-      <c r="B37">
-        <v>0.0027498017162912278</v>
-      </c>
-      <c r="C37" t="s">
-        <v>14</v>
-      </c>
-      <c r="D37">
-        <v>0</v>
-      </c>
-      <c r="E37">
-        <v>0</v>
-      </c>
-      <c r="F37">
-        <v>0</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-      <c r="H37">
-        <v>0.03336996655614665</v>
-      </c>
-      <c r="I37">
-        <v>0</v>
-      </c>
-      <c r="J37">
-        <v>0</v>
-      </c>
-      <c r="K37">
-        <v>0</v>
-      </c>
-      <c r="L37">
-        <v>0</v>
-      </c>
-      <c r="M37">
-        <v>0.0052647563328623529</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="s">
-        <v>52</v>
       </c>
       <c r="B38">
         <v>0.64065857495279754</v>
       </c>
       <c r="C38" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D38">
         <v>0.62735855600145474</v>
@@ -2594,15 +2306,15 @@
         <v>0.65282270441129442</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B39">
         <v>0.13178127675598383</v>
       </c>
       <c r="C39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D39">
         <v>0.17392665539625113</v>
@@ -2611,7 +2323,7 @@
         <v>0.14999999999999997</v>
       </c>
       <c r="F39">
-        <v>0.075960626071199994</v>
+        <v>7.5960626071199994E-2</v>
       </c>
       <c r="G39">
         <v>0</v>
@@ -2632,18 +2344,18 @@
         <v>0.19293812597000576</v>
       </c>
       <c r="M39">
-        <v>0.093235328533420231</v>
-      </c>
-    </row>
-    <row r="40">
+        <v>9.3235328533420231E-2</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B40">
-        <v>0.033525704932213241</v>
+        <v>3.3525704932213241E-2</v>
       </c>
       <c r="C40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D40">
         <v>0</v>
@@ -2655,7 +2367,7 @@
         <v>0.16153217810996306</v>
       </c>
       <c r="G40">
-        <v>0.083495776591012316</v>
+        <v>8.3495776591012316E-2</v>
       </c>
       <c r="H40">
         <v>0</v>
@@ -2667,65 +2379,65 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K40">
-        <v>0.04697960827488723</v>
+        <v>4.697960827488723E-2</v>
       </c>
       <c r="L40">
-        <v>0.076391784051418346</v>
+        <v>7.6391784051418346E-2</v>
       </c>
       <c r="M40">
-        <v>0.064188143570440226</v>
-      </c>
-    </row>
-    <row r="41">
+        <v>6.4188143570440226E-2</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>54</v>
+      </c>
+      <c r="B41">
+        <v>1.0093356468659548E-2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41">
+        <v>0</v>
+      </c>
+      <c r="E41">
+        <v>7.4663247585067358E-2</v>
+      </c>
+      <c r="F41">
+        <v>0</v>
+      </c>
+      <c r="G41">
+        <v>0</v>
+      </c>
+      <c r="H41">
+        <v>4.989010033156005E-2</v>
+      </c>
+      <c r="I41">
+        <v>0</v>
+      </c>
+      <c r="J41">
+        <v>0</v>
+      </c>
+      <c r="K41">
+        <v>0</v>
+      </c>
+      <c r="L41">
+        <v>0</v>
+      </c>
+      <c r="M41">
+        <v>1.9324688785154816E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>55</v>
-      </c>
-      <c r="B41">
-        <v>0.010093356468659548</v>
-      </c>
-      <c r="C41" t="s">
-        <v>14</v>
-      </c>
-      <c r="D41">
-        <v>0</v>
-      </c>
-      <c r="E41">
-        <v>0.074663247585067358</v>
-      </c>
-      <c r="F41">
-        <v>0</v>
-      </c>
-      <c r="G41">
-        <v>0</v>
-      </c>
-      <c r="H41">
-        <v>0.04989010033156005</v>
-      </c>
-      <c r="I41">
-        <v>0</v>
-      </c>
-      <c r="J41">
-        <v>0</v>
-      </c>
-      <c r="K41">
-        <v>0</v>
-      </c>
-      <c r="L41">
-        <v>0</v>
-      </c>
-      <c r="M41">
-        <v>0.019324688785154816</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="s">
-        <v>56</v>
       </c>
       <c r="B42">
         <v>0.25209298365274435</v>
       </c>
       <c r="C42" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D42">
         <v>0.17675660161956802</v>
@@ -2740,7 +2452,7 @@
         <v>0.2877920415082113</v>
       </c>
       <c r="H42">
-        <v>0.052937832745001252</v>
+        <v>5.2937832745001252E-2</v>
       </c>
       <c r="I42">
         <v>0</v>
@@ -2758,15 +2470,15 @@
         <v>0.32099525419378022</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B43">
         <v>0.24473096466009769</v>
       </c>
       <c r="C43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D43">
         <v>0.31422396551346782</v>
@@ -2799,15 +2511,15 @@
         <v>0.18117302072540334</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B44">
         <v>0.77814961510638658</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D44">
         <v>0.77942946215406539</v>
@@ -2840,15 +2552,15 @@
         <v>0.77697907352806306</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B45">
         <v>0.80058154951358007</v>
       </c>
       <c r="C45" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D45">
         <v>0.86539996799781638</v>
@@ -2881,15 +2593,15 @@
         <v>0.74129895475775365</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B46">
         <v>0.34700986924206628</v>
       </c>
       <c r="C46" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D46">
         <v>0.2250517404111412</v>
@@ -2922,15 +2634,15 @@
         <v>0.45855215147810913</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B47">
         <v>0.16598392458026229</v>
       </c>
       <c r="C47" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D47">
         <v>0.18871308729812913</v>
@@ -2939,13 +2651,13 @@
         <v>0.34134541318423095</v>
       </c>
       <c r="F47">
-        <v>0.037877172753991946</v>
+        <v>3.7877172753991946E-2</v>
       </c>
       <c r="G47">
         <v>0.18658477958201991</v>
       </c>
       <c r="H47">
-        <v>0.092335050210445038</v>
+        <v>9.2335050210445038E-2</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -2954,7 +2666,7 @@
         <v>0</v>
       </c>
       <c r="K47">
-        <v>0.093624470070135302</v>
+        <v>9.3624470070135302E-2</v>
       </c>
       <c r="L47">
         <v>0.14999999999999986</v>
@@ -2963,15 +2675,15 @@
         <v>0.14519594835294602</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B48">
         <v>0.1919665423499598</v>
       </c>
       <c r="C48" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D48">
         <v>0.13597076653851345</v>
@@ -2983,7 +2695,7 @@
         <v>0.1735862451682324</v>
       </c>
       <c r="G48">
-        <v>0.0502282515626283</v>
+        <v>5.02282515626283E-2</v>
       </c>
       <c r="H48">
         <v>0.47673812465953469</v>
@@ -2998,21 +2710,21 @@
         <v>0.56502682522727088</v>
       </c>
       <c r="L48">
-        <v>0.049999999999999947</v>
+        <v>4.9999999999999947E-2</v>
       </c>
       <c r="M48">
         <v>0.24317999314212016</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B49">
         <v>0.21031349165515134</v>
       </c>
       <c r="C49" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D49">
         <v>0.25471912760544407</v>
@@ -3024,7 +2736,7 @@
         <v>0.2112304355910555</v>
       </c>
       <c r="G49">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H49">
         <v>0</v>
@@ -3045,18 +2757,18 @@
         <v>0.16970032363168</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B50">
         <v>0.16591045502041432</v>
       </c>
       <c r="C50" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D50">
-        <v>0.089596947104695221</v>
+        <v>8.9596947104695221E-2</v>
       </c>
       <c r="E50">
         <v>0.57636626686972681</v>
@@ -3065,7 +2777,7 @@
         <v>0.11383779882519193</v>
       </c>
       <c r="G50">
-        <v>0.052734174689060394</v>
+        <v>5.2734174689060394E-2</v>
       </c>
       <c r="H50">
         <v>0</v>
@@ -3086,30 +2798,30 @@
         <v>0.2357063999070268</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B51">
-        <v>0.08327285797182167</v>
+        <v>8.327285797182167E-2</v>
       </c>
       <c r="C51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D51">
-        <v>0.028535961053762403</v>
+        <v>2.8535961053762403E-2</v>
       </c>
       <c r="E51">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="F51">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="G51">
         <v>0.15986286393554253</v>
       </c>
       <c r="H51">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="I51">
         <v>0.5</v>
@@ -3127,15 +2839,15 @@
         <v>0.13333494455256606</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B52">
         <v>0.19394215906571266</v>
       </c>
       <c r="C52" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D52">
         <v>0.2619063667562207</v>
@@ -3147,10 +2859,10 @@
         <v>0.12560119787250951</v>
       </c>
       <c r="G52">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="H52">
-        <v>0.01764594424833375</v>
+        <v>1.764594424833375E-2</v>
       </c>
       <c r="I52">
         <v>0</v>
@@ -3159,7 +2871,7 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K52">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L52">
         <v>0.40938151411569101</v>
@@ -3168,15 +2880,15 @@
         <v>0.13178244155583413</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53">
         <v>0.51958980428657342</v>
       </c>
       <c r="C53" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D53">
         <v>0.57025133966324293</v>
@@ -3188,7 +2900,7 @@
         <v>0.4534587792127327</v>
       </c>
       <c r="G53">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="H53">
         <v>0.83288915102041261</v>
@@ -3197,7 +2909,7 @@
         <v>0</v>
       </c>
       <c r="J53">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K53">
         <v>0.24721605430452737</v>
@@ -3209,24 +2921,24 @@
         <v>0.4732550225736647</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B54">
         <v>0.17364709658904501</v>
       </c>
       <c r="C54" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D54">
         <v>0.16515743435259284</v>
       </c>
       <c r="E54">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F54">
-        <v>0.088150348306102966</v>
+        <v>8.8150348306102966E-2</v>
       </c>
       <c r="G54">
         <v>0.1466793202632774</v>
@@ -3241,24 +2953,24 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K54">
-        <v>0.078187764964932335</v>
+        <v>7.8187764964932335E-2</v>
       </c>
       <c r="L54">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M54">
         <v>0.18141169834494622</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B55">
         <v>0.22105093552249797</v>
       </c>
       <c r="C55" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D55">
         <v>0.18855443247764755</v>
@@ -3291,56 +3003,56 @@
         <v>0.25077207136690099</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>70</v>
+      </c>
+      <c r="B56">
+        <v>0</v>
+      </c>
+      <c r="C56" t="s">
+        <v>13</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>0</v>
+      </c>
+      <c r="G56">
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>0</v>
+      </c>
+      <c r="I56">
+        <v>0</v>
+      </c>
+      <c r="J56">
+        <v>0</v>
+      </c>
+      <c r="K56">
+        <v>0</v>
+      </c>
+      <c r="L56">
+        <v>0</v>
+      </c>
+      <c r="M56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
         <v>71</v>
-      </c>
-      <c r="B56">
-        <v>0</v>
-      </c>
-      <c r="C56" t="s">
-        <v>14</v>
-      </c>
-      <c r="D56">
-        <v>0</v>
-      </c>
-      <c r="E56">
-        <v>0</v>
-      </c>
-      <c r="F56">
-        <v>0</v>
-      </c>
-      <c r="G56">
-        <v>0</v>
-      </c>
-      <c r="H56">
-        <v>0</v>
-      </c>
-      <c r="I56">
-        <v>0</v>
-      </c>
-      <c r="J56">
-        <v>0</v>
-      </c>
-      <c r="K56">
-        <v>0</v>
-      </c>
-      <c r="L56">
-        <v>0</v>
-      </c>
-      <c r="M56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="s">
-        <v>72</v>
       </c>
       <c r="B57">
         <v>0.47290674879984573</v>
       </c>
       <c r="C57" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D57">
         <v>0.36411941303303608</v>
@@ -3373,15 +3085,15 @@
         <v>0.57240309091436758</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B58">
         <v>0.18051421639542869</v>
       </c>
       <c r="C58" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D58">
         <v>0.1216576931116455</v>
@@ -3390,13 +3102,13 @@
         <v>0.67981880223653623</v>
       </c>
       <c r="F58">
-        <v>0.013120807626654752</v>
+        <v>1.3120807626654752E-2</v>
       </c>
       <c r="G58">
         <v>0.17578058229686799</v>
       </c>
       <c r="H58">
-        <v>0.01764594424833375</v>
+        <v>1.764594424833375E-2</v>
       </c>
       <c r="I58">
         <v>0</v>
@@ -3414,15 +3126,15 @@
         <v>0.23434409222644656</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B59">
         <v>0.33069517139195903</v>
       </c>
       <c r="C59" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D59">
         <v>0.30763403084422319</v>
@@ -3449,24 +3161,24 @@
         <v>0.56445309651650399</v>
       </c>
       <c r="L59">
-        <v>0.076391784051418346</v>
+        <v>7.6391784051418346E-2</v>
       </c>
       <c r="M59">
         <v>0.35178677284828064</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B60">
         <v>0.12172476719532502</v>
       </c>
       <c r="C60" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D60">
-        <v>0.065402522105664745</v>
+        <v>6.5402522105664745E-2</v>
       </c>
       <c r="E60">
         <v>0.59520045497345997</v>
@@ -3478,7 +3190,7 @@
         <v>0</v>
       </c>
       <c r="H60">
-        <v>0.067536044579893803</v>
+        <v>6.7536044579893803E-2</v>
       </c>
       <c r="I60">
         <v>0.5</v>
@@ -3490,21 +3202,21 @@
         <v>0.21173811612731119</v>
       </c>
       <c r="L60">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M60">
         <v>0.17323680512325895</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B61">
         <v>0.26916550253504357</v>
       </c>
       <c r="C61" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D61">
         <v>0.32885156888621181</v>
@@ -3516,7 +3228,7 @@
         <v>0.14951423774633407</v>
       </c>
       <c r="G61">
-        <v>0.097106123203848302</v>
+        <v>9.7106123203848302E-2</v>
       </c>
       <c r="H61">
         <v>0.14528809894100228</v>
@@ -3531,71 +3243,71 @@
         <v>0.66970046866354505</v>
       </c>
       <c r="L61">
-        <v>0.02546392801713945</v>
+        <v>2.546392801713945E-2</v>
       </c>
       <c r="M61">
         <v>0.21457693084802837</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>76</v>
+      </c>
+      <c r="B62">
+        <v>4.970205662625881E-2</v>
+      </c>
+      <c r="C62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D62">
+        <v>0.05</v>
+      </c>
+      <c r="E62">
+        <v>0.05</v>
+      </c>
+      <c r="F62">
+        <v>0.05</v>
+      </c>
+      <c r="G62">
+        <v>0.05</v>
+      </c>
+      <c r="H62">
+        <v>0.05</v>
+      </c>
+      <c r="I62">
+        <v>0</v>
+      </c>
+      <c r="J62">
+        <v>4.1666666666666657E-2</v>
+      </c>
+      <c r="K62">
+        <v>4.6868026115007511E-2</v>
+      </c>
+      <c r="L62">
+        <v>4.9999999999999947E-2</v>
+      </c>
+      <c r="M62">
+        <v>4.9429559137138826E-2</v>
+      </c>
+    </row>
+    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
         <v>77</v>
       </c>
-      <c r="B62">
-        <v>0.04970205662625881</v>
-      </c>
-      <c r="C62" t="s">
-        <v>14</v>
-      </c>
-      <c r="D62">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="E62">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="F62">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="G62">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="H62">
-        <v>0.050000000000000003</v>
-      </c>
-      <c r="I62">
-        <v>0</v>
-      </c>
-      <c r="J62">
-        <v>0.041666666666666657</v>
-      </c>
-      <c r="K62">
-        <v>0.046868026115007511</v>
-      </c>
-      <c r="L62">
-        <v>0.049999999999999947</v>
-      </c>
-      <c r="M62">
-        <v>0.049429559137138826</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="s">
-        <v>78</v>
-      </c>
       <c r="B63">
-        <v>0.094741047573845896</v>
+        <v>9.4741047573845896E-2</v>
       </c>
       <c r="C63" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D63">
-        <v>0.057722628867841803</v>
+        <v>5.7722628867841803E-2</v>
       </c>
       <c r="E63">
         <v>0.42596376044730722</v>
       </c>
       <c r="F63">
-        <v>0.039362422879964276</v>
+        <v>3.9362422879964276E-2</v>
       </c>
       <c r="G63">
         <v>0</v>
@@ -3610,7 +3322,7 @@
         <v>0.12499999999999997</v>
       </c>
       <c r="K63">
-        <v>0.046979608274887237</v>
+        <v>4.6979608274887237E-2</v>
       </c>
       <c r="L63">
         <v>0.14999999999999986</v>
@@ -3619,15 +3331,15 @@
         <v>0.12859790440510691</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B64">
-        <v>0.084347716177630747</v>
+        <v>8.4347716177630747E-2</v>
       </c>
       <c r="C64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -3654,21 +3366,21 @@
         <v>0.198733331358149</v>
       </c>
       <c r="L64">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M64">
         <v>0.16149170693936207</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B65">
         <v>0.14919547511559123</v>
       </c>
       <c r="C65" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D65">
         <v>0.18350063969479294</v>
@@ -3695,30 +3407,30 @@
         <v>0</v>
       </c>
       <c r="L65">
-        <v>0.073608215948581496</v>
+        <v>7.3608215948581496E-2</v>
       </c>
       <c r="M65">
         <v>0.11782014666206933</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B66">
         <v>0.14953695378717047</v>
       </c>
       <c r="C66" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D66">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="E66">
         <v>0.36345413184230912</v>
       </c>
       <c r="F66">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="G66">
         <v>0</v>
@@ -3742,27 +3454,27 @@
         <v>0.14911345408399479</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B67">
         <v>0.11233098484112555</v>
       </c>
       <c r="C67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D67">
-        <v>0.093816194227781924</v>
+        <v>9.3816194227781924E-2</v>
       </c>
       <c r="E67">
         <v>0.14999999999999997</v>
       </c>
       <c r="F67">
-        <v>0.075960626071199994</v>
+        <v>7.5960626071199994E-2</v>
       </c>
       <c r="G67">
-        <v>0.052734174689060394</v>
+        <v>5.2734174689060394E-2</v>
       </c>
       <c r="H67">
         <v>0.23376408928484957</v>
@@ -3783,56 +3495,56 @@
         <v>0.12926451784898144</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>82</v>
+      </c>
+      <c r="B68">
+        <v>4.3903212000548641E-2</v>
+      </c>
+      <c r="C68" t="s">
+        <v>13</v>
+      </c>
+      <c r="D68">
+        <v>2.8535961053762403E-2</v>
+      </c>
+      <c r="E68">
+        <v>2.5112250804977549E-2</v>
+      </c>
+      <c r="F68">
+        <v>7.7239595633956201E-2</v>
+      </c>
+      <c r="G68">
+        <v>0</v>
+      </c>
+      <c r="H68">
+        <v>6.7536044579893803E-2</v>
+      </c>
+      <c r="I68">
+        <v>0</v>
+      </c>
+      <c r="J68">
+        <v>0</v>
+      </c>
+      <c r="K68">
+        <v>9.3624470070135302E-2</v>
+      </c>
+      <c r="L68">
+        <v>7.6391784051418346E-2</v>
+      </c>
+      <c r="M68">
+        <v>5.7958021292308461E-2</v>
+      </c>
+    </row>
+    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
         <v>83</v>
-      </c>
-      <c r="B68">
-        <v>0.043903212000548641</v>
-      </c>
-      <c r="C68" t="s">
-        <v>14</v>
-      </c>
-      <c r="D68">
-        <v>0.028535961053762403</v>
-      </c>
-      <c r="E68">
-        <v>0.025112250804977549</v>
-      </c>
-      <c r="F68">
-        <v>0.077239595633956201</v>
-      </c>
-      <c r="G68">
-        <v>0</v>
-      </c>
-      <c r="H68">
-        <v>0.067536044579893803</v>
-      </c>
-      <c r="I68">
-        <v>0</v>
-      </c>
-      <c r="J68">
-        <v>0</v>
-      </c>
-      <c r="K68">
-        <v>0.093624470070135302</v>
-      </c>
-      <c r="L68">
-        <v>0.076391784051418346</v>
-      </c>
-      <c r="M68">
-        <v>0.057958021292308461</v>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="s">
-        <v>84</v>
       </c>
       <c r="B69">
         <v>0.6250199960014442</v>
       </c>
       <c r="C69" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D69">
         <v>0.47895265719717645</v>
@@ -3865,27 +3577,27 @@
         <v>0.75861243864182348</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B70">
         <v>0.12962216344211727</v>
       </c>
       <c r="C70" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D70">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="E70">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F70">
         <v>0.144017014604292</v>
       </c>
       <c r="G70">
-        <v>0.097265825310939594</v>
+        <v>9.7265825310939594E-2</v>
       </c>
       <c r="H70">
         <v>0.127050798588003</v>
@@ -3906,15 +3618,15 @@
         <v>0.11098469812112638</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B71">
         <v>0.79255711980158061</v>
       </c>
       <c r="C71" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D71">
         <v>0.77352222364879752</v>
@@ -3947,27 +3659,27 @@
         <v>0.809966338681537</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B72">
         <v>0.20622978576125026</v>
       </c>
       <c r="C72" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D72">
         <v>0.19097949547488646</v>
       </c>
       <c r="E72">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F72">
         <v>0.16689594740282954</v>
       </c>
       <c r="G72">
-        <v>0.063780324269187394</v>
+        <v>6.3780324269187394E-2</v>
       </c>
       <c r="H72">
         <v>0.61760863119074094</v>
@@ -3988,15 +3700,15 @@
         <v>0.22017762342987671</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B73">
         <v>0.45659819675080326</v>
       </c>
       <c r="C73" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D73">
         <v>0.44624074733523938</v>
@@ -4029,30 +3741,30 @@
         <v>0.46607106712878354</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B74">
-        <v>0.042908168280703554</v>
+        <v>4.2908168280703554E-2</v>
       </c>
       <c r="C74" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D74">
         <v>0</v>
       </c>
       <c r="E74">
-        <v>0.025112250804977549</v>
+        <v>2.5112250804977549E-2</v>
       </c>
       <c r="F74">
         <v>0.11340179680876425</v>
       </c>
       <c r="G74">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="H74">
-        <v>0.03336996655614665</v>
+        <v>3.336996655614665E-2</v>
       </c>
       <c r="I74">
         <v>0</v>
@@ -4067,18 +3779,18 @@
         <v>0.14999999999999986</v>
       </c>
       <c r="M74">
-        <v>0.082151760015642061</v>
-      </c>
-    </row>
-    <row r="75">
+        <v>8.2151760015642061E-2</v>
+      </c>
+    </row>
+    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B75">
         <v>0.64625677245233759</v>
       </c>
       <c r="C75" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D75">
         <v>0.65732566090682809</v>
@@ -4111,18 +3823,18 @@
         <v>0.6361332235600643</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B76">
         <v>0.16339811885445843</v>
       </c>
       <c r="C76" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D76">
-        <v>0.094219936801335447</v>
+        <v>9.4219936801335447E-2</v>
       </c>
       <c r="E76">
         <v>0.14999999999999997</v>
@@ -4140,10 +3852,10 @@
         <v>0</v>
       </c>
       <c r="J76">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K76">
-        <v>0.076972782749568314</v>
+        <v>7.6972782749568314E-2</v>
       </c>
       <c r="L76">
         <v>0.14999999999999986</v>
@@ -4152,56 +3864,56 @@
         <v>0.22666813112107143</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>91</v>
+      </c>
+      <c r="B77">
+        <v>0</v>
+      </c>
+      <c r="C77" t="s">
+        <v>13</v>
+      </c>
+      <c r="D77">
+        <v>0</v>
+      </c>
+      <c r="E77">
+        <v>0</v>
+      </c>
+      <c r="F77">
+        <v>0</v>
+      </c>
+      <c r="G77">
+        <v>0</v>
+      </c>
+      <c r="H77">
+        <v>0</v>
+      </c>
+      <c r="I77">
+        <v>0</v>
+      </c>
+      <c r="J77">
+        <v>0</v>
+      </c>
+      <c r="K77">
+        <v>0</v>
+      </c>
+      <c r="L77">
+        <v>0</v>
+      </c>
+      <c r="M77">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
         <v>92</v>
       </c>
-      <c r="B77">
-        <v>0</v>
-      </c>
-      <c r="C77" t="s">
-        <v>14</v>
-      </c>
-      <c r="D77">
-        <v>0</v>
-      </c>
-      <c r="E77">
-        <v>0</v>
-      </c>
-      <c r="F77">
-        <v>0</v>
-      </c>
-      <c r="G77">
-        <v>0</v>
-      </c>
-      <c r="H77">
-        <v>0</v>
-      </c>
-      <c r="I77">
-        <v>0</v>
-      </c>
-      <c r="J77">
-        <v>0</v>
-      </c>
-      <c r="K77">
-        <v>0</v>
-      </c>
-      <c r="L77">
-        <v>0</v>
-      </c>
-      <c r="M77">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="s">
-        <v>93</v>
-      </c>
       <c r="B78">
-        <v>0.077367366622963438</v>
+        <v>7.7367366622963438E-2</v>
       </c>
       <c r="C78" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D78">
         <v>0.16195931755638138</v>
@@ -4234,15 +3946,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B79">
         <v>0.2110655966013123</v>
       </c>
       <c r="C79" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D79">
         <v>0.1917943011483639</v>
@@ -4254,7 +3966,7 @@
         <v>0.10149306375597081</v>
       </c>
       <c r="G79">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H79">
         <v>0.17854816582870897</v>
@@ -4269,21 +3981,21 @@
         <v>0.27703616021030264</v>
       </c>
       <c r="L79">
-        <v>0.076391784051418346</v>
+        <v>7.6391784051418346E-2</v>
       </c>
       <c r="M79">
         <v>0.22869102507477598</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B80">
         <v>0.6934289354872627</v>
       </c>
       <c r="C80" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D80">
         <v>0.5057008628898092</v>
@@ -4316,15 +4028,15 @@
         <v>0.86512407264636793</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B81">
         <v>0.40868702900587339</v>
       </c>
       <c r="C81" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D81">
         <v>0.25989486782691623</v>
@@ -4357,15 +4069,15 @@
         <v>0.54477158028447248</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B82">
         <v>0.13351841569318368</v>
       </c>
       <c r="C82" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D82">
         <v>0.13411230558546383</v>
@@ -4374,13 +4086,13 @@
         <v>0.14999999999999997</v>
       </c>
       <c r="F82">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="G82">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H82">
-        <v>0.052937832745001252</v>
+        <v>5.2937832745001252E-2</v>
       </c>
       <c r="I82">
         <v>0</v>
@@ -4398,56 +4110,56 @@
         <v>0.13297524702852107</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>97</v>
+      </c>
+      <c r="B83">
+        <v>0</v>
+      </c>
+      <c r="C83" t="s">
+        <v>13</v>
+      </c>
+      <c r="D83">
+        <v>0</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>0</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>0</v>
+      </c>
+      <c r="I83">
+        <v>0</v>
+      </c>
+      <c r="J83">
+        <v>0</v>
+      </c>
+      <c r="K83">
+        <v>0</v>
+      </c>
+      <c r="L83">
+        <v>0</v>
+      </c>
+      <c r="M83">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
         <v>98</v>
-      </c>
-      <c r="B83">
-        <v>0</v>
-      </c>
-      <c r="C83" t="s">
-        <v>14</v>
-      </c>
-      <c r="D83">
-        <v>0</v>
-      </c>
-      <c r="E83">
-        <v>0</v>
-      </c>
-      <c r="F83">
-        <v>0</v>
-      </c>
-      <c r="G83">
-        <v>0</v>
-      </c>
-      <c r="H83">
-        <v>0</v>
-      </c>
-      <c r="I83">
-        <v>0</v>
-      </c>
-      <c r="J83">
-        <v>0</v>
-      </c>
-      <c r="K83">
-        <v>0</v>
-      </c>
-      <c r="L83">
-        <v>0</v>
-      </c>
-      <c r="M83">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="s">
-        <v>99</v>
       </c>
       <c r="B84">
         <v>0.84278302241396652</v>
       </c>
       <c r="C84" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D84">
         <v>0.78593522219628187</v>
@@ -4480,56 +4192,56 @@
         <v>0.89477573037990987</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>99</v>
+      </c>
+      <c r="B85">
+        <v>0</v>
+      </c>
+      <c r="C85" t="s">
+        <v>13</v>
+      </c>
+      <c r="D85">
+        <v>0</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>0</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>0</v>
+      </c>
+      <c r="I85">
+        <v>0</v>
+      </c>
+      <c r="J85">
+        <v>0</v>
+      </c>
+      <c r="K85">
+        <v>0</v>
+      </c>
+      <c r="L85">
+        <v>0</v>
+      </c>
+      <c r="M85">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
         <v>100</v>
-      </c>
-      <c r="B85">
-        <v>0</v>
-      </c>
-      <c r="C85" t="s">
-        <v>14</v>
-      </c>
-      <c r="D85">
-        <v>0</v>
-      </c>
-      <c r="E85">
-        <v>0</v>
-      </c>
-      <c r="F85">
-        <v>0</v>
-      </c>
-      <c r="G85">
-        <v>0</v>
-      </c>
-      <c r="H85">
-        <v>0</v>
-      </c>
-      <c r="I85">
-        <v>0</v>
-      </c>
-      <c r="J85">
-        <v>0</v>
-      </c>
-      <c r="K85">
-        <v>0</v>
-      </c>
-      <c r="L85">
-        <v>0</v>
-      </c>
-      <c r="M85">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="s">
-        <v>101</v>
       </c>
       <c r="B86">
         <v>0.24689553598701525</v>
       </c>
       <c r="C86" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D86">
         <v>0.25043692982022259</v>
@@ -4562,27 +4274,27 @@
         <v>0.24365659526006939</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B87">
-        <v>0.090826691489049025</v>
+        <v>9.0826691489049025E-2</v>
       </c>
       <c r="C87" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D87">
-        <v>0.048663077244658216</v>
+        <v>4.8663077244658216E-2</v>
       </c>
       <c r="E87">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="F87">
         <v>0.10149306375597081</v>
       </c>
       <c r="G87">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="H87">
         <v>0.16633566639321973</v>
@@ -4597,21 +4309,21 @@
         <v>0.35409112507272006</v>
       </c>
       <c r="L87">
-        <v>0.02546392801713945</v>
+        <v>2.546392801713945E-2</v>
       </c>
       <c r="M87">
         <v>0.12938931790208172</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B88">
         <v>0.66432413227573628</v>
       </c>
       <c r="C88" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D88">
         <v>0.83773882202862782</v>
@@ -4644,27 +4356,27 @@
         <v>0.50571994202033477</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B89">
-        <v>0.079518375502701327</v>
+        <v>7.9518375502701327E-2</v>
       </c>
       <c r="C89" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D89">
-        <v>0.07457531793850132</v>
+        <v>7.457531793850132E-2</v>
       </c>
       <c r="E89">
         <v>0.25452854661909424</v>
       </c>
       <c r="F89">
-        <v>0.07552462405477231</v>
+        <v>7.552462405477231E-2</v>
       </c>
       <c r="G89">
-        <v>0.083495776591012316</v>
+        <v>8.3495776591012316E-2</v>
       </c>
       <c r="H89">
         <v>0</v>
@@ -4676,24 +4388,24 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K89">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L89">
         <v>0</v>
       </c>
       <c r="M89">
-        <v>0.084039270724858894</v>
-      </c>
-    </row>
-    <row r="90">
+        <v>8.4039270724858894E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B90">
         <v>0.50739422507905307</v>
       </c>
       <c r="C90" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D90">
         <v>0.58112639629353779</v>
@@ -4714,36 +4426,36 @@
         <v>0</v>
       </c>
       <c r="J90">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K90">
-        <v>0.046868026115007511</v>
+        <v>4.6868026115007511E-2</v>
       </c>
       <c r="L90">
-        <v>0.049999999999999947</v>
+        <v>4.9999999999999947E-2</v>
       </c>
       <c r="M90">
         <v>0.43995915756597348</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B91">
-        <v>0.018837650039502819</v>
+        <v>1.8837650039502819E-2</v>
       </c>
       <c r="C91" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D91">
         <v>0</v>
       </c>
       <c r="E91">
-        <v>0.025112250804977549</v>
+        <v>2.5112250804977549E-2</v>
       </c>
       <c r="F91">
-        <v>0.069977640675492017</v>
+        <v>6.9977640675492017E-2</v>
       </c>
       <c r="G91">
         <v>0</v>
@@ -4764,18 +4476,18 @@
         <v>0</v>
       </c>
       <c r="M91">
-        <v>0.036066468630865336</v>
-      </c>
-    </row>
-    <row r="92">
+        <v>3.6066468630865336E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B92">
         <v>0.49702056626258806</v>
       </c>
       <c r="C92" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D92">
         <v>0.5</v>
@@ -4808,30 +4520,30 @@
         <v>0.49429559137138829</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B93">
         <v>0.10659115973726827</v>
       </c>
       <c r="C93" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D93">
         <v>0.11350269206650634</v>
       </c>
       <c r="E93">
-        <v>0.074663247585067344</v>
+        <v>7.4663247585067344E-2</v>
       </c>
       <c r="F93">
-        <v>0.077239595633956201</v>
+        <v>7.7239595633956201E-2</v>
       </c>
       <c r="G93">
         <v>0.10296242625168869</v>
       </c>
       <c r="H93">
-        <v>0.052937832745001252</v>
+        <v>5.2937832745001252E-2</v>
       </c>
       <c r="I93">
         <v>0</v>
@@ -4849,15 +4561,15 @@
         <v>0.10026990754078557</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B94">
         <v>0.2588690766028966</v>
       </c>
       <c r="C94" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D94">
         <v>0.16172065765150223</v>
@@ -4869,7 +4581,7 @@
         <v>0.18683163346356502</v>
       </c>
       <c r="G94">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H94">
         <v>0.5036631082916182</v>
@@ -4890,15 +4602,15 @@
         <v>0.34772052479528653</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B95">
         <v>0.33121087789314985</v>
       </c>
       <c r="C95" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D95">
         <v>0</v>
@@ -4931,56 +4643,56 @@
         <v>0.63413465653542511</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>110</v>
+      </c>
+      <c r="B96">
+        <v>0</v>
+      </c>
+      <c r="C96" t="s">
+        <v>13</v>
+      </c>
+      <c r="D96">
+        <v>0</v>
+      </c>
+      <c r="E96">
+        <v>0</v>
+      </c>
+      <c r="F96">
+        <v>0</v>
+      </c>
+      <c r="G96">
+        <v>0</v>
+      </c>
+      <c r="H96">
+        <v>0</v>
+      </c>
+      <c r="I96">
+        <v>0</v>
+      </c>
+      <c r="J96">
+        <v>0</v>
+      </c>
+      <c r="K96">
+        <v>0</v>
+      </c>
+      <c r="L96">
+        <v>0</v>
+      </c>
+      <c r="M96">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
         <v>111</v>
       </c>
-      <c r="B96">
-        <v>0</v>
-      </c>
-      <c r="C96" t="s">
-        <v>14</v>
-      </c>
-      <c r="D96">
-        <v>0</v>
-      </c>
-      <c r="E96">
-        <v>0</v>
-      </c>
-      <c r="F96">
-        <v>0</v>
-      </c>
-      <c r="G96">
-        <v>0</v>
-      </c>
-      <c r="H96">
-        <v>0</v>
-      </c>
-      <c r="I96">
-        <v>0</v>
-      </c>
-      <c r="J96">
-        <v>0</v>
-      </c>
-      <c r="K96">
-        <v>0</v>
-      </c>
-      <c r="L96">
-        <v>0</v>
-      </c>
-      <c r="M96">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" t="s">
-        <v>112</v>
-      </c>
       <c r="B97">
-        <v>0.049992306679587636</v>
+        <v>4.9992306679587636E-2</v>
       </c>
       <c r="C97" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D97">
         <v>0</v>
@@ -4989,7 +4701,7 @@
         <v>0.32851828937429634</v>
       </c>
       <c r="F97">
-        <v>0.036598203191235745</v>
+        <v>3.6598203191235745E-2</v>
       </c>
       <c r="G97">
         <v>0</v>
@@ -5004,27 +4716,27 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K97">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L97">
         <v>0</v>
       </c>
       <c r="M97">
-        <v>0.095715015241441159</v>
-      </c>
-    </row>
-    <row r="98">
+        <v>9.5715015241441159E-2</v>
+      </c>
+    </row>
+    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B98">
-        <v>0.072920558992630308</v>
+        <v>7.2920558992630308E-2</v>
       </c>
       <c r="C98" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D98">
-        <v>0.049110575227793551</v>
+        <v>4.9110575227793551E-2</v>
       </c>
       <c r="E98">
         <v>0.61730917363153814</v>
@@ -5051,18 +4763,18 @@
         <v>0</v>
       </c>
       <c r="M98">
-        <v>0.094697048633717501</v>
-      </c>
-    </row>
-    <row r="99">
+        <v>9.4697048633717501E-2</v>
+      </c>
+    </row>
+    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B99">
         <v>0.11518713936974463</v>
       </c>
       <c r="C99" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D99">
         <v>0</v>
@@ -5095,15 +4807,15 @@
         <v>0.22053670919919344</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B100">
-        <v>0.037127654295618144</v>
+        <v>3.7127654295618144E-2</v>
       </c>
       <c r="C100" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D100">
         <v>0</v>
@@ -5115,7 +4827,7 @@
         <v>0.11340179680876425</v>
       </c>
       <c r="G100">
-        <v>0.14999999999999999</v>
+        <v>0.15</v>
       </c>
       <c r="H100">
         <v>0</v>
@@ -5133,18 +4845,18 @@
         <v>0</v>
       </c>
       <c r="M100">
-        <v>0.07108441743967478</v>
-      </c>
-    </row>
-    <row r="101">
+        <v>7.108441743967478E-2</v>
+      </c>
+    </row>
+    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B101">
         <v>0.75314996527822164</v>
       </c>
       <c r="C101" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D101">
         <v>0.77466374817774475</v>
@@ -5177,27 +4889,27 @@
         <v>0.73347356923027685</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B102">
-        <v>0.038082848904222519</v>
+        <v>3.8082848904222519E-2</v>
       </c>
       <c r="C102" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D102">
-        <v>0.030154337451012501</v>
+        <v>3.0154337451012501E-2</v>
       </c>
       <c r="E102">
-        <v>0.02488774919502245</v>
+        <v>2.488774919502245E-2</v>
       </c>
       <c r="F102">
-        <v>0.025746531877985403</v>
+        <v>2.5746531877985403E-2</v>
       </c>
       <c r="G102">
-        <v>0.032421941770313205</v>
+        <v>3.2421941770313205E-2</v>
       </c>
       <c r="H102">
         <v>0.14528809894100228</v>
@@ -5206,27 +4918,27 @@
         <v>0</v>
       </c>
       <c r="J102">
-        <v>0.041666666666666657</v>
+        <v>4.1666666666666657E-2</v>
       </c>
       <c r="K102">
-        <v>0.046868026115007511</v>
+        <v>4.6868026115007511E-2</v>
       </c>
       <c r="L102">
         <v>0</v>
       </c>
       <c r="M102">
-        <v>0.045334225017508716</v>
-      </c>
-    </row>
-    <row r="103">
+        <v>4.5334225017508716E-2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B103">
         <v>0.38114579548428562</v>
       </c>
       <c r="C103" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D103">
         <v>0.50385609686325328</v>
@@ -5235,10 +4947,10 @@
         <v>0</v>
       </c>
       <c r="F103">
-        <v>0.0509979803806467</v>
+        <v>5.09979803806467E-2</v>
       </c>
       <c r="G103">
-        <v>0.0502282515626283</v>
+        <v>5.02282515626283E-2</v>
       </c>
       <c r="H103">
         <v>0.79864850528291176</v>
@@ -5259,27 +4971,27 @@
         <v>0.26891558007438865</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B104">
         <v>0.13980139723378857</v>
       </c>
       <c r="C104" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D104">
-        <v>0.01637019174259785</v>
+        <v>1.637019174259785E-2</v>
       </c>
       <c r="E104">
         <v>0.59520045497345997</v>
       </c>
       <c r="F104">
-        <v>0.051988147131294925</v>
+        <v>5.1988147131294925E-2</v>
       </c>
       <c r="G104">
-        <v>0.083495776591012316</v>
+        <v>8.3495776591012316E-2</v>
       </c>
       <c r="H104">
         <v>0.33842007353115044</v>
@@ -5300,24 +5012,24 @@
         <v>0.25269094786571233</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B105">
-        <v>0.084013816820461731</v>
+        <v>8.4013816820461731E-2</v>
       </c>
       <c r="C105" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D105">
-        <v>0.02303967971346885</v>
+        <v>2.303967971346885E-2</v>
       </c>
       <c r="E105">
         <v>0.25452854661909424</v>
       </c>
       <c r="F105">
-        <v>0.076241615253309511</v>
+        <v>7.6241615253309511E-2</v>
       </c>
       <c r="G105">
         <v>0.1148438835406264</v>
@@ -5341,15 +5053,15 @@
         <v>0.1397804514473025</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B106">
         <v>0.24905665126647203</v>
       </c>
       <c r="C106" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D106">
         <v>0.14550749349071351</v>
@@ -5361,7 +5073,7 @@
         <v>0.49493437621946967</v>
       </c>
       <c r="G106">
-        <v>0.032421941770313205</v>
+        <v>3.2421941770313205E-2</v>
       </c>
       <c r="H106">
         <v>0.56552713295507251</v>
@@ -5382,21 +5094,21 @@
         <v>0.34376218252253549</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B107">
         <v>0.25693649875121949</v>
       </c>
       <c r="C107" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D107">
         <v>0.21376994646760566</v>
       </c>
       <c r="E107">
-        <v>0.050000000000000003</v>
+        <v>0.05</v>
       </c>
       <c r="F107">
         <v>0.65821745773463136</v>
@@ -5423,15 +5135,15 @@
         <v>0.29641640717660062</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B108">
         <v>0.55550210202440409</v>
       </c>
       <c r="C108" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D108">
         <v>0.4120586285318863</v>
@@ -5464,15 +5176,15 @@
         <v>0.6866947708411103</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B109">
         <v>0.21480467756508889</v>
       </c>
       <c r="C109" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D109">
         <v>0.23644162404551294</v>
@@ -5487,7 +5199,7 @@
         <v>0.12656563872247278</v>
       </c>
       <c r="H109">
-        <v>0.069291806016055627</v>
+        <v>6.9291806016055627E-2</v>
       </c>
       <c r="I109">
         <v>0</v>
@@ -5505,15 +5217,15 @@
         <v>0.19501563673459665</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B110">
-        <v>0.053870973424069407</v>
+        <v>5.3870973424069407E-2</v>
       </c>
       <c r="C110" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D110">
         <v>0.11277243200456297</v>
@@ -5546,15 +5258,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B111">
-        <v>0.024689008618535423</v>
+        <v>2.4689008618535423E-2</v>
       </c>
       <c r="C111" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D111">
         <v>0</v>
@@ -5569,7 +5281,7 @@
         <v>0</v>
       </c>
       <c r="H111">
-        <v>0.077642154692668511</v>
+        <v>7.7642154692668511E-2</v>
       </c>
       <c r="I111">
         <v>0</v>
@@ -5584,18 +5296,18 @@
         <v>0</v>
       </c>
       <c r="M111">
-        <v>0.04726944990486049</v>
-      </c>
-    </row>
-    <row r="112">
+        <v>4.726944990486049E-2</v>
+      </c>
+    </row>
+    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B112">
         <v>0.38307939602900959</v>
       </c>
       <c r="C112" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D112">
         <v>0.30836105942830827</v>
@@ -5628,30 +5340,30 @@
         <v>0.45141640537159433</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B113">
-        <v>0.062578175517364332</v>
+        <v>6.2578175517364332E-2</v>
       </c>
       <c r="C113" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D113">
-        <v>0.03649730793349365</v>
+        <v>3.649730793349365E-2</v>
       </c>
       <c r="E113">
-        <v>0.075336752414932637</v>
+        <v>7.5336752414932637E-2</v>
       </c>
       <c r="F113">
         <v>0.11212282724600806</v>
       </c>
       <c r="G113">
-        <v>0.099771748437371688</v>
+        <v>9.9771748437371688E-2</v>
       </c>
       <c r="H113">
-        <v>0.052937832745001252</v>
+        <v>5.2937832745001252E-2</v>
       </c>
       <c r="I113">
         <v>0</v>
@@ -5660,65 +5372,65 @@
         <v>0.12499999999999994</v>
       </c>
       <c r="K113">
-        <v>0.095446943393181327</v>
+        <v>9.5446943393181327E-2</v>
       </c>
       <c r="L113">
-        <v>0.076391784051418346</v>
+        <v>7.6391784051418346E-2</v>
       </c>
       <c r="M113">
-        <v>0.086431603910267787</v>
-      </c>
-    </row>
-    <row r="114">
+        <v>8.6431603910267787E-2</v>
+      </c>
+    </row>
+    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
+        <v>127</v>
+      </c>
+      <c r="B114">
+        <v>1.6610422941708509E-2</v>
+      </c>
+      <c r="C114" t="s">
+        <v>13</v>
+      </c>
+      <c r="D114">
+        <v>0</v>
+      </c>
+      <c r="E114">
+        <v>2.488774919502245E-2</v>
+      </c>
+      <c r="F114">
+        <v>0</v>
+      </c>
+      <c r="G114">
+        <v>0</v>
+      </c>
+      <c r="H114">
+        <v>6.9291806016055627E-2</v>
+      </c>
+      <c r="I114">
+        <v>0</v>
+      </c>
+      <c r="J114">
+        <v>0</v>
+      </c>
+      <c r="K114">
+        <v>9.3624470070135302E-2</v>
+      </c>
+      <c r="L114">
+        <v>0</v>
+      </c>
+      <c r="M114">
+        <v>3.1802230995705838E-2</v>
+      </c>
+    </row>
+    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
         <v>128</v>
-      </c>
-      <c r="B114">
-        <v>0.016610422941708509</v>
-      </c>
-      <c r="C114" t="s">
-        <v>14</v>
-      </c>
-      <c r="D114">
-        <v>0</v>
-      </c>
-      <c r="E114">
-        <v>0.02488774919502245</v>
-      </c>
-      <c r="F114">
-        <v>0</v>
-      </c>
-      <c r="G114">
-        <v>0</v>
-      </c>
-      <c r="H114">
-        <v>0.069291806016055627</v>
-      </c>
-      <c r="I114">
-        <v>0</v>
-      </c>
-      <c r="J114">
-        <v>0</v>
-      </c>
-      <c r="K114">
-        <v>0.093624470070135302</v>
-      </c>
-      <c r="L114">
-        <v>0</v>
-      </c>
-      <c r="M114">
-        <v>0.031802230995705838</v>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="s">
-        <v>129</v>
       </c>
       <c r="B115">
         <v>0.80732705955737716</v>
       </c>
       <c r="C115" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D115">
         <v>0.84608458821144894</v>
@@ -5751,15 +5463,15 @@
         <v>0.77187962164286761</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B116">
         <v>0.49350037577294892</v>
       </c>
       <c r="C116" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D116">
         <v>0.43315685465374953</v>
@@ -5793,9 +5505,7 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait"/>
 </worksheet>
 </file>
</xml_diff>